<commit_message>
Maisons de gestion renseignées sur 11 fiches, benchmark retiré de la fiche 34 ; audit recalculé
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VZYZDQZsmCyRopyNrtR5g1
</commit_message>
<xml_diff>
--- a/docs/2026-10-13-audit-documents.xlsx
+++ b/docs/2026-10-13-audit-documents.xlsx
@@ -434,13 +434,11 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Audit des documents des fiches invest-law.eu — calcul sur le site le 14/10/2026 à 09h41 UTC (461 fiches de fonds externes)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+          <t>Audit des documents des fiches invest-law.eu — calcul sur le site le 14/10/2026 à 09h51 UTC (461 fiches de fonds externes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -483,9 +481,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -623,13 +619,11 @@
           <t>ALKEN SMALL CAP EUROPE</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>aucune</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -650,13 +644,16 @@
           <t>Smart Value Investors - Patrimoine Flexible A Acc</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Conventum</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>aucune</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -722,7 +719,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -753,7 +749,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -784,7 +779,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -815,7 +809,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -916,7 +909,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>Aucune factsheet (seulement un rapport annuel ou semestriel)</t>
@@ -982,7 +974,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -1118,7 +1109,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -1149,7 +1139,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -1180,7 +1169,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -1246,7 +1234,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -1487,7 +1474,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>Aucune factsheet (seulement un rapport annuel ou semestriel)</t>
@@ -1588,7 +1574,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -1619,7 +1604,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -1685,7 +1669,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -1751,7 +1734,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -1782,7 +1764,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -1988,7 +1969,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -2054,7 +2034,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
           <t>Aucune factsheet (seulement un rapport annuel ou semestriel)</t>
@@ -2085,7 +2064,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -2116,7 +2094,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -2147,7 +2124,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -2248,7 +2224,6 @@
           <t>aucune</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
           <t>Aucune factsheet</t>
@@ -2516,13 +2491,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -3183,13 +3156,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -3310,13 +3281,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -3482,13 +3451,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -3529,7 +3496,6 @@
           <t>FR</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -4910,13 +4876,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -4992,13 +4956,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -5254,13 +5216,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -6506,13 +6466,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -6553,7 +6511,6 @@
           <t>FR</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -6854,13 +6811,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -11121,13 +11076,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G197" t="inlineStr"/>
       <c r="H197" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -11168,7 +11121,6 @@
           <t>FR</t>
         </is>
       </c>
-      <c r="I198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -11244,13 +11196,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G200" t="inlineStr"/>
       <c r="H200" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -11291,7 +11241,6 @@
           <t>FR</t>
         </is>
       </c>
-      <c r="I201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -11817,13 +11766,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G213" t="inlineStr"/>
       <c r="H213" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -11944,13 +11891,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G216" t="inlineStr"/>
       <c r="H216" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -12026,13 +11971,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G218" t="inlineStr"/>
       <c r="H218" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -14268,13 +14211,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G268" t="inlineStr"/>
       <c r="H268" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -14440,13 +14381,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G272" t="inlineStr"/>
       <c r="H272" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -14522,13 +14461,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G274" t="inlineStr"/>
       <c r="H274" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -14604,13 +14541,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G276" t="inlineStr"/>
       <c r="H276" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="n">
@@ -14686,13 +14621,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G278" t="inlineStr"/>
       <c r="H278" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="n">
@@ -14768,13 +14701,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G280" t="inlineStr"/>
       <c r="H280" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="n">
@@ -14850,13 +14781,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G282" t="inlineStr"/>
       <c r="H282" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="n">
@@ -14932,13 +14861,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G284" t="inlineStr"/>
       <c r="H284" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="n">
@@ -15014,13 +14941,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G286" t="inlineStr"/>
       <c r="H286" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="n">
@@ -15096,13 +15021,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G288" t="inlineStr"/>
       <c r="H288" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="n">
@@ -15268,13 +15191,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G292" t="inlineStr"/>
       <c r="H292" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="n">
@@ -15305,13 +15226,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G293" t="inlineStr"/>
       <c r="H293" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="n">
@@ -15387,13 +15306,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G295" t="inlineStr"/>
       <c r="H295" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="n">
@@ -15784,13 +15701,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G304" t="inlineStr"/>
       <c r="H304" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="n">
@@ -15866,13 +15781,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G306" t="inlineStr"/>
       <c r="H306" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="n">
@@ -15948,13 +15861,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G308" t="inlineStr"/>
       <c r="H308" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="n">
@@ -16390,13 +16301,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G318" t="inlineStr"/>
       <c r="H318" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="n">
@@ -16517,13 +16426,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G321" t="inlineStr"/>
       <c r="H321" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="n">
@@ -16599,13 +16506,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G323" t="inlineStr"/>
       <c r="H323" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="n">
@@ -16681,13 +16586,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G325" t="inlineStr"/>
       <c r="H325" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="n">
@@ -16763,13 +16666,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G327" t="inlineStr"/>
       <c r="H327" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="n">
@@ -16845,13 +16746,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G329" t="inlineStr"/>
       <c r="H329" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="n">
@@ -16972,13 +16871,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G332" t="inlineStr"/>
       <c r="H332" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="n">
@@ -17099,13 +16996,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G335" t="inlineStr"/>
       <c r="H335" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="n">
@@ -17181,13 +17076,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G337" t="inlineStr"/>
       <c r="H337" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="n">
@@ -17263,13 +17156,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G339" t="inlineStr"/>
       <c r="H339" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="n">
@@ -17345,13 +17236,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G341" t="inlineStr"/>
       <c r="H341" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="n">
@@ -17427,13 +17316,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G343" t="inlineStr"/>
       <c r="H343" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="n">
@@ -17509,13 +17396,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G345" t="inlineStr"/>
       <c r="H345" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="n">
@@ -17591,13 +17476,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G347" t="inlineStr"/>
       <c r="H347" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="n">
@@ -17673,13 +17556,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G349" t="inlineStr"/>
       <c r="H349" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="n">
@@ -17755,13 +17636,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G351" t="inlineStr"/>
       <c r="H351" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="n">
@@ -17837,13 +17716,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G353" t="inlineStr"/>
       <c r="H353" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="n">
@@ -17919,13 +17796,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G355" t="inlineStr"/>
       <c r="H355" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="n">
@@ -18001,13 +17876,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G357" t="inlineStr"/>
       <c r="H357" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="n">
@@ -18128,13 +18001,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G360" t="inlineStr"/>
       <c r="H360" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="n">
@@ -18255,13 +18126,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G363" t="inlineStr"/>
       <c r="H363" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="n">
@@ -18382,13 +18251,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G366" t="inlineStr"/>
       <c r="H366" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="n">
@@ -18509,13 +18376,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G369" t="inlineStr"/>
       <c r="H369" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="n">
@@ -18636,13 +18501,11 @@
           <t>DIC</t>
         </is>
       </c>
-      <c r="G372" t="inlineStr"/>
       <c r="H372" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="n">
@@ -18773,7 +18636,6 @@
           <t>FR</t>
         </is>
       </c>
-      <c r="I375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="n">
@@ -25114,7 +24976,6 @@
           <t>FR</t>
         </is>
       </c>
-      <c r="I516" t="inlineStr"/>
     </row>
     <row r="517">
       <c r="A517" t="n">
@@ -25290,7 +25151,6 @@
           <t>FR</t>
         </is>
       </c>
-      <c r="I520" t="inlineStr"/>
     </row>
     <row r="521">
       <c r="A521" t="n">
@@ -26681,7 +26541,6 @@
           <t>EN</t>
         </is>
       </c>
-      <c r="I551" t="inlineStr"/>
     </row>
     <row r="552">
       <c r="A552" t="n">
@@ -28342,7 +28201,6 @@
           <t>EN</t>
         </is>
       </c>
-      <c r="I588" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" t="n">
@@ -28428,7 +28286,6 @@
           <t>EN</t>
         </is>
       </c>
-      <c r="I590" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" t="n">
@@ -28514,7 +28371,6 @@
           <t>EN</t>
         </is>
       </c>
-      <c r="I592" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" t="n">

</xml_diff>